<commit_message>
Predict days from the estimated delivery date and align regression with classification
- Target: delivery date minus estimated delivery date (negative = early),
  with the lead time still capped at 45 days
- Same section order and names as model_classification_dev.ipynb
- Same split: 335 training days and a 30-day hold-out, no gap before it;
  CV folds keep the 45-day gap
- Champion chosen by hold-out MAE, at the main run date and at each
  backtest run date
- Uses the shared make_preprocessor
- Regenerated figures, tuning JSON and report tables

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/phase2/results/regression_report_tables.xlsx
+++ b/phase2/results/regression_report_tables.xlsx
@@ -515,6 +515,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -547,7 +548,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Lead time in days from approval to delivery, capped at 45 days</t>
+          <t>Days from the estimated delivery date (negative = early, positive = late); lead time capped at 45 days</t>
         </is>
       </c>
     </row>
@@ -559,7 +560,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>LightGBM (tuned), CV MAE 6.117 days</t>
+          <t>LightGBM (tuned), lowest hold-out MAE (5.847 days; CV MAE 5.624)</t>
         </is>
       </c>
     </row>
@@ -575,6 +576,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
@@ -607,7 +609,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Distribution of lead time for delivered orders (all of 2017-2018)</t>
+          <t>Distribution of lead time and days from promise for delivered orders (all of 2017-2018)</t>
         </is>
       </c>
     </row>
@@ -619,7 +621,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Chronological split of the 2018-06-02 training window (2017-10-20 to 2018-04-17)</t>
+          <t>Chronological split of the 2018-06-02 training window (2017-04-18 to 2018-04-17)</t>
         </is>
       </c>
     </row>
@@ -679,7 +681,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Hold-out evaluation on the newest 45 approval days (2018-03-04 to 2018-04-17)</t>
+          <t>Hold-out evaluation on the newest 30 approval days (2018-03-19 to 2018-04-17)</t>
         </is>
       </c>
     </row>
@@ -867,7 +869,7 @@
         </is>
       </c>
       <c r="E3" s="8" t="n">
-        <v>7.921229704541891</v>
+        <v>6.837064070902182</v>
       </c>
       <c r="F3" s="10" t="n"/>
     </row>
@@ -888,13 +890,13 @@
         </is>
       </c>
       <c r="D4" s="13" t="n">
-        <v>1000</v>
+        <v>0.08111308307896872</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>7.851365385831554</v>
+        <v>6.812111238922651</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>7.466878292203377</v>
+        <v>6.670931265188512</v>
       </c>
     </row>
     <row r="5">
@@ -917,10 +919,10 @@
         <v>200</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>8.748025436598647</v>
+        <v>8.642644390013142</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>6.403964535538281</v>
+        <v>5.912638205795114</v>
       </c>
     </row>
     <row r="6">
@@ -943,10 +945,10 @@
         <v>12</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>8.748025436598647</v>
+        <v>8.642644390013142</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>6.403964535538281</v>
+        <v>5.912638205795114</v>
       </c>
     </row>
     <row r="7">
@@ -969,10 +971,10 @@
         <v>200</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>6.342097338399386</v>
+        <v>5.885218329668307</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>6.231352929827908</v>
+        <v>5.708676430383172</v>
       </c>
     </row>
     <row r="8">
@@ -992,13 +994,13 @@
         </is>
       </c>
       <c r="D8" s="13" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>6.342097338399386</v>
+        <v>5.885218329668307</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>6.231352929827908</v>
+        <v>5.708676430383172</v>
       </c>
     </row>
     <row r="9">
@@ -1018,13 +1020,13 @@
         </is>
       </c>
       <c r="D9" s="13" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>6.342097338399386</v>
+        <v>5.885218329668307</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>6.231352929827908</v>
+        <v>5.708676430383172</v>
       </c>
     </row>
     <row r="10">
@@ -1044,13 +1046,13 @@
         </is>
       </c>
       <c r="D10" s="13" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>6.342097338399386</v>
+        <v>5.885218329668307</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>6.231352929827908</v>
+        <v>5.708676430383172</v>
       </c>
     </row>
     <row r="11">
@@ -1073,10 +1075,10 @@
         <v>1</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>6.24728877605728</v>
+        <v>5.751597282021803</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>6.116957743249393</v>
+        <v>5.623849362046951</v>
       </c>
     </row>
     <row r="12">
@@ -1096,13 +1098,13 @@
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>6.24728877605728</v>
+        <v>5.751597282021803</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>6.116957743249393</v>
+        <v>5.623849362046951</v>
       </c>
     </row>
     <row r="13">
@@ -1127,10 +1129,10 @@
         </is>
       </c>
       <c r="E13" s="8" t="n">
-        <v>6.24728877605728</v>
+        <v>5.751597282021803</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>6.116957743249393</v>
+        <v>5.623849362046951</v>
       </c>
     </row>
     <row r="14">
@@ -1150,13 +1152,13 @@
         </is>
       </c>
       <c r="D14" s="13" t="n">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>6.24728877605728</v>
+        <v>5.751597282021803</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>6.116957743249393</v>
+        <v>5.623849362046951</v>
       </c>
     </row>
     <row r="15">
@@ -1179,10 +1181,10 @@
         <v>600</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>6.24728877605728</v>
+        <v>5.751597282021803</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>6.116957743249393</v>
+        <v>5.623849362046951</v>
       </c>
     </row>
     <row r="16">
@@ -1202,13 +1204,13 @@
         </is>
       </c>
       <c r="D16" s="13" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>6.24728877605728</v>
+        <v>5.751597282021803</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>6.116957743249393</v>
+        <v>5.623849362046951</v>
       </c>
     </row>
     <row r="17">
@@ -1228,13 +1230,13 @@
         </is>
       </c>
       <c r="D17" s="13" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>6.24728877605728</v>
+        <v>5.751597282021803</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>6.116957743249393</v>
+        <v>5.623849362046951</v>
       </c>
     </row>
     <row r="18">
@@ -1254,13 +1256,13 @@
         </is>
       </c>
       <c r="D18" s="13" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>6.24728877605728</v>
+        <v>5.751597282021803</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>6.116957743249393</v>
+        <v>5.623849362046951</v>
       </c>
     </row>
     <row r="19">
@@ -1338,19 +1340,19 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>6367</v>
+        <v>4109</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>18.279</v>
+        <v>-10.104</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>17.255</v>
+        <v>-8.352</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>-1.024</v>
+        <v>1.752</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>7.495</v>
+        <v>7.205</v>
       </c>
     </row>
     <row r="4">
@@ -1360,19 +1362,19 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>3891</v>
+        <v>2715</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>8.087</v>
+        <v>-9.207000000000001</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>7.351</v>
+        <v>-8.94</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>-0.736</v>
+        <v>0.267</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>3.848</v>
+        <v>3.813</v>
       </c>
     </row>
     <row r="5">
@@ -1382,28 +1384,30 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>6.481</v>
+        <v>-18.957</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>7.656</v>
+        <v>-16.321</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.174</v>
+        <v>2.635</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>3.063</v>
+        <v>3.294</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Note: Bias = mean(predicted - actual).</t>
-        </is>
-      </c>
-    </row>
+          <t>Note: Actual and predicted are days from the promised date (negative = early). Bias = mean(predicted - actual).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -1450,19 +1454,19 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>4450</v>
+        <v>3071</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>9.025</v>
+        <v>-9.821</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>8.387</v>
+        <v>-9.211</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>-0.638</v>
+        <v>0.611</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>4.119</v>
+        <v>4.101</v>
       </c>
     </row>
     <row r="12">
@@ -1472,19 +1476,19 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>1270</v>
+        <v>798</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>20.527</v>
+        <v>-12.006</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>19.996</v>
+        <v>-8.954000000000001</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>-0.531</v>
+        <v>3.052</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>9.927</v>
+        <v>9.728</v>
       </c>
     </row>
     <row r="13">
@@ -1494,19 +1498,19 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>1224</v>
+        <v>782</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>14.708</v>
+        <v>-10.514</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>13.316</v>
+        <v>-8.983000000000001</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>-1.392</v>
+        <v>1.531</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>6.176</v>
+        <v>5.629</v>
       </c>
     </row>
     <row r="14">
@@ -1516,19 +1520,19 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>570</v>
+        <v>382</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>17.918</v>
+        <v>-12.047</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>17.368</v>
+        <v>-9.369999999999999</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>-0.549</v>
+        <v>2.677</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>7.233</v>
+        <v>6.887</v>
       </c>
     </row>
     <row r="15">
@@ -1538,107 +1542,107 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>543</v>
+        <v>363</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>12.996</v>
+        <v>-12.102</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>12.939</v>
+        <v>-9.829000000000001</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>-0.058</v>
+        <v>2.273</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>5.333</v>
+        <v>5.295</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>353</v>
+        <v>225</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>22.686</v>
+        <v>-10.884</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>19.135</v>
+        <v>-7.013</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>-3.551</v>
+        <v>3.871</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>8.24</v>
+        <v>6.447</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>341</v>
+        <v>219</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>15.038</v>
+        <v>-4.402</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>17.232</v>
+        <v>-5.56</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>2.194</v>
+        <v>-1.158</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>6.233</v>
+        <v>7.536</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>206</v>
+        <v>144</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>14.437</v>
+        <v>-4.583</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>16.055</v>
+        <v>-5.967</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>1.618</v>
+        <v>-1.384</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>6.331</v>
+        <v>6.358</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>202</v>
+        <v>139</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>19.98</v>
+        <v>-10.367</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>17.051</v>
+        <v>-6.296</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>-2.93</v>
+        <v>4.071</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>7.419</v>
+        <v>6.082</v>
       </c>
     </row>
     <row r="20">
@@ -1648,19 +1652,19 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>200</v>
+        <v>121</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>18.08</v>
+        <v>-8.24</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>17.634</v>
+        <v>-6.622</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>-0.446</v>
+        <v>1.618</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>6.526</v>
+        <v>5.99</v>
       </c>
     </row>
     <row r="21">
@@ -1670,19 +1674,19 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>160</v>
+        <v>105</v>
       </c>
       <c r="C21" s="8" t="n">
-        <v>20.606</v>
+        <v>-7.543</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>19.021</v>
+        <v>-7.381</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>-1.585</v>
+        <v>0.162</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>7.697</v>
+        <v>7.559</v>
       </c>
     </row>
     <row r="22">
@@ -1692,19 +1696,19 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>147</v>
+        <v>100</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>26.993</v>
+        <v>-1.92</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>23.818</v>
+        <v>-2.991</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>-3.175</v>
+        <v>-1.071</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>9.446999999999999</v>
+        <v>9.477</v>
       </c>
     </row>
     <row r="23">
@@ -1725,7 +1729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1758,30 +1762,25 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Balanced accuracy</t>
+          <t>Precision</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>Precision</t>
+          <t>Recall</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Recall</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>ROC-AUC</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>ROC-AUC</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>PR-AUC</t>
         </is>
@@ -1794,25 +1793,22 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>0.851</v>
+        <v>0.896</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>0.539</v>
+        <v>0.432</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>0.579</v>
+        <v>0.106</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>0.089</v>
+        <v>0.17</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>0.155</v>
+        <v>0.707</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>0.698</v>
-      </c>
-      <c r="H3" s="8" t="n">
-        <v>0.337</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="4">
@@ -1822,25 +1818,22 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>0.439</v>
+        <v>0.414</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>0.613</v>
+        <v>0.128</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>0.196</v>
+        <v>0.832</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>0.863</v>
+        <v>0.222</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.319</v>
+        <v>0.676</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>0.256</v>
+        <v>0.208</v>
       </c>
     </row>
     <row r="5">
@@ -1850,25 +1843,22 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>0.711</v>
+        <v>0.673</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>0.632</v>
+        <v>0.185</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>0.268</v>
+        <v>0.662</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>0.518</v>
+        <v>0.29</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.353</v>
+        <v>0.705</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>0.669</v>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>0.252</v>
+        <v>0.208</v>
       </c>
     </row>
     <row r="6">
@@ -1878,25 +1868,22 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>0.587</v>
+        <v>0.391</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>0.656</v>
+        <v>0.132</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0.234</v>
+        <v>0.907</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>0.755</v>
+        <v>0.231</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.357</v>
+        <v>0.732</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>0.723</v>
-      </c>
-      <c r="H6" s="8" t="n">
-        <v>0.332</v>
+        <v>0.239</v>
       </c>
     </row>
     <row r="7">
@@ -1906,31 +1893,28 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>0.696</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>0.668</v>
+        <v>0.158</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>0.279</v>
+        <v>0.784</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>0.628</v>
+        <v>0.263</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.386</v>
+        <v>0.741</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.723</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>0.335</v>
+        <v>0.259</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Note: Regression-derived flag: predicted lead time &gt; promised lead time. Classifiers use a 0.5 threshold. Hold-out late rate: 15.23%. "v2 features" = the base classification feature set.</t>
+          <t>Note: Regression-derived flag: predicted days from the promised date &gt; 0. Classifiers use a 0.5 threshold. Hold-out late rate: 10.06%. "v2 features" = the base classification feature set.</t>
         </is>
       </c>
     </row>
@@ -1945,17 +1929,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2006,31 +1991,39 @@
           <t>Lowest target-known %</t>
         </is>
       </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Max capped before promise %</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
         <v>21</v>
       </c>
       <c r="B3" s="8" t="n">
-        <v>12.94</v>
+        <v>12.54</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>15.57</v>
+        <v>13.65</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>19.77</v>
+        <v>15.74</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>16.46</v>
+        <v>14.94</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>12.94</v>
+        <v>12.54</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>19.77</v>
+        <v>15.74</v>
       </c>
       <c r="H3" s="8" t="n">
-        <v>99.97</v>
+        <v>99.98</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>13.09</v>
       </c>
     </row>
     <row r="4">
@@ -2038,25 +2031,28 @@
         <v>30</v>
       </c>
       <c r="B4" s="8" t="n">
-        <v>5.9</v>
+        <v>5.91</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>6.82</v>
+        <v>6.17</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>9.09</v>
+        <v>7.22</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>7.38</v>
+        <v>6.73</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>5.9</v>
+        <v>5.91</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>9.09</v>
+        <v>7.22</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>99.97</v>
+        <v>99.98</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>2.41</v>
       </c>
     </row>
     <row r="5">
@@ -2064,38 +2060,43 @@
         <v>45</v>
       </c>
       <c r="B5" s="8" t="n">
-        <v>2.7</v>
+        <v>3.04</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>2.82</v>
+        <v>2.92</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>3.47</v>
+        <v>3.11</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>2.94</v>
+        <v>2.83</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>2.7</v>
+        <v>2.83</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>3.47</v>
+        <v>3.11</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>99.97</v>
+        <v>99.98</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Note: Capped % = orders delivered after the cap or still undelivered at the cap. Each run date uses its own 180-day window ending 45 days before the inference date. Min and Max are taken over the four run dates.</t>
-        </is>
-      </c>
-    </row>
+          <t>Note: Capped % = orders delivered after the cap or still undelivered at the cap. Each run date uses its own 365-day window ending 45 days before the inference date. Min and Max are taken over the four run dates. Capped before promise = capped orders whose promised lead time is longer than the cap, so they are recorded as early.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Distribution of lead time for delivered orders (all of 2017-2018)</t>
+          <t>Distribution of lead time and days from promise for delivered orders (all of 2017-2018)</t>
         </is>
       </c>
     </row>
@@ -2110,6 +2111,11 @@
           <t>Lead days (delivered orders)</t>
         </is>
       </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Days from promise (delivered orders)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -2120,6 +2126,9 @@
       <c r="B11" s="8" t="n">
         <v>96190</v>
       </c>
+      <c r="C11" s="8" t="n">
+        <v>96190</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -2130,6 +2139,9 @@
       <c r="B12" s="8" t="n">
         <v>11.965</v>
       </c>
+      <c r="C12" s="8" t="n">
+        <v>-11.806</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -2140,6 +2152,9 @@
       <c r="B13" s="8" t="n">
         <v>9.51</v>
       </c>
+      <c r="C13" s="8" t="n">
+        <v>10.089</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -2150,6 +2165,9 @@
       <c r="B14" s="8" t="n">
         <v>-7</v>
       </c>
+      <c r="C14" s="8" t="n">
+        <v>-147</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -2160,6 +2178,9 @@
       <c r="B15" s="8" t="n">
         <v>10</v>
       </c>
+      <c r="C15" s="8" t="n">
+        <v>-12</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -2170,6 +2191,9 @@
       <c r="B16" s="8" t="n">
         <v>15</v>
       </c>
+      <c r="C16" s="8" t="n">
+        <v>-7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -2180,6 +2204,9 @@
       <c r="B17" s="8" t="n">
         <v>22</v>
       </c>
+      <c r="C17" s="8" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -2190,6 +2217,9 @@
       <c r="B18" s="8" t="n">
         <v>29</v>
       </c>
+      <c r="C18" s="8" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -2200,6 +2230,9 @@
       <c r="B19" s="8" t="n">
         <v>45</v>
       </c>
+      <c r="C19" s="8" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -2210,11 +2243,14 @@
       <c r="B20" s="8" t="n">
         <v>208</v>
       </c>
+      <c r="C20" s="8" t="n">
+        <v>188</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Note: Days from approval to customer delivery, before capping.</t>
+          <t>Note: Lead days = approval to customer delivery, before capping. Days from promise = delivery date - estimated delivery date (negative = early).</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2279,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Chronological split of the 2018-06-02 training window (2017-10-20 to 2018-04-17)</t>
+          <t>Chronological split of the 2018-06-02 training window (2017-04-18 to 2018-04-17)</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2306,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Mean capped lead days</t>
+          <t>Mean days from promise</t>
         </is>
       </c>
     </row>
@@ -2282,19 +2318,19 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>2017-10-20</t>
+          <t>2017-04-18</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>2018-03-03</t>
+          <t>2018-03-18</t>
         </is>
       </c>
       <c r="D3" s="7" t="n">
-        <v>29247</v>
+        <v>55994</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>14.86</v>
+        <v>-10.6</v>
       </c>
     </row>
     <row r="4">
@@ -2305,7 +2341,7 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>2018-03-04</t>
+          <t>2018-03-19</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
@@ -2314,19 +2350,21 @@
         </is>
       </c>
       <c r="D4" s="7" t="n">
-        <v>10285</v>
+        <v>6847</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>14.39</v>
+        <v>-9.779999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Note: The hold-out is the newest 45 approval days.</t>
-        </is>
-      </c>
-    </row>
+          <t>Note: The hold-out is the newest 30 approval days. Training uses every earlier approval day in the window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
@@ -2362,7 +2400,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Validation mean capped lead days</t>
+          <t>Validation mean days from promise</t>
         </is>
       </c>
     </row>
@@ -2371,23 +2409,23 @@
         <v>1</v>
       </c>
       <c r="B10" s="7" t="n">
-        <v>3307</v>
+        <v>4920</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>6602</v>
+        <v>6631</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>2017-11-12</t>
+          <t>2017-07-17</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>2017-12-04</t>
+          <t>2017-09-03</t>
         </is>
       </c>
       <c r="F10" s="8" t="n">
-        <v>15.46</v>
+        <v>-12.34</v>
       </c>
     </row>
     <row r="11">
@@ -2395,23 +2433,23 @@
         <v>2</v>
       </c>
       <c r="B11" s="7" t="n">
-        <v>9909</v>
+        <v>10579</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>4354</v>
+        <v>7151</v>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>2017-12-05</t>
+          <t>2017-09-04</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>2017-12-27</t>
+          <t>2017-10-22</t>
         </is>
       </c>
       <c r="F11" s="8" t="n">
-        <v>15.09</v>
+        <v>-11.26</v>
       </c>
     </row>
     <row r="12">
@@ -2419,23 +2457,23 @@
         <v>3</v>
       </c>
       <c r="B12" s="7" t="n">
-        <v>14263</v>
+        <v>17137</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>4676</v>
+        <v>11010</v>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>2017-12-28</t>
+          <t>2017-10-23</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>2018-01-18</t>
+          <t>2017-12-10</t>
         </is>
       </c>
       <c r="F12" s="8" t="n">
-        <v>13.57</v>
+        <v>-8.9</v>
       </c>
     </row>
     <row r="13">
@@ -2443,23 +2481,23 @@
         <v>4</v>
       </c>
       <c r="B13" s="7" t="n">
-        <v>18939</v>
+        <v>24334</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>4954</v>
+        <v>9717</v>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>2018-01-19</t>
+          <t>2017-12-11</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>2018-02-09</t>
+          <t>2018-01-28</t>
         </is>
       </c>
       <c r="F13" s="8" t="n">
-        <v>14.72</v>
+        <v>-13.1</v>
       </c>
     </row>
     <row r="14">
@@ -2467,29 +2505,29 @@
         <v>5</v>
       </c>
       <c r="B14" s="7" t="n">
-        <v>23893</v>
+        <v>35686</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>5354</v>
+        <v>11554</v>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>2018-02-10</t>
+          <t>2018-01-29</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>2018-03-03</t>
+          <t>2018-03-18</t>
         </is>
       </c>
       <c r="F14" s="8" t="n">
-        <v>16.9</v>
+        <v>-7.38</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Note: Each fold trains on all approval days before its validation block.</t>
+          <t>Note: Each fold trains on approval days up to 45 days before its validation block, using outcomes known at that point.</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2593,7 @@
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>Baseline: predicts the training median</t>
+          <t>Baseline: predicts the training median days from promise</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
@@ -2577,7 +2615,7 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Baseline: Olist's promised lead time, capped at 45 days</t>
+          <t>Baseline: delivery exactly on the promised date (zero days off)</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
@@ -2810,22 +2848,22 @@
         </is>
       </c>
       <c r="E3" s="12" t="n">
-        <v>6.117</v>
+        <v>5.624</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>0.573</v>
+        <v>0.974</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>9.244</v>
+        <v>8.856</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>0.853</v>
+        <v>1.062</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.183</v>
+        <v>0.098</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>0.08</v>
+        <v>0.08500000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -2844,24 +2882,24 @@
           <t>Tree-based</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr"/>
+      <c r="D4" s="10" t="n"/>
       <c r="E4" s="8" t="n">
-        <v>6.231</v>
+        <v>5.709</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.435</v>
+        <v>0.897</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>8.914999999999999</v>
+        <v>8.693</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>0.728</v>
+        <v>1.086</v>
       </c>
       <c r="I4" s="8" t="n">
-        <v>0.24</v>
+        <v>0.133</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>0.062</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -2880,24 +2918,24 @@
           <t>Tree-based</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr"/>
+      <c r="D5" s="10" t="n"/>
       <c r="E5" s="8" t="n">
-        <v>6.247</v>
+        <v>5.752</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.476</v>
+        <v>0.877</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>8.944000000000001</v>
+        <v>8.622999999999999</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>0.733</v>
+        <v>1.043</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>0.235</v>
+        <v>0.145</v>
       </c>
       <c r="J5" s="8" t="n">
-        <v>0.059</v>
+        <v>0.08400000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -2916,24 +2954,24 @@
           <t>Tree-based</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr"/>
+      <c r="D6" s="10" t="n"/>
       <c r="E6" s="8" t="n">
-        <v>6.342</v>
+        <v>5.885</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.427</v>
+        <v>0.917</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>9.003</v>
+        <v>8.675000000000001</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>0.725</v>
+        <v>1.038</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>0.225</v>
+        <v>0.135</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>0.058</v>
+        <v>0.082</v>
       </c>
     </row>
     <row r="7">
@@ -2952,96 +2990,96 @@
           <t>Tree-based</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr"/>
+      <c r="D7" s="10" t="n"/>
       <c r="E7" s="8" t="n">
-        <v>6.404</v>
+        <v>5.913</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.443</v>
+        <v>0.918</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>9.164</v>
+        <v>8.84</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>0.736</v>
+        <v>1.068</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.196</v>
+        <v>0.102</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>0.066</v>
+        <v>0.076</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>Dummy (median)</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Linear</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr"/>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n"/>
       <c r="E8" s="8" t="n">
-        <v>7.467</v>
+        <v>6.586</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>1.553</v>
+        <v>1.036</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>10.004</v>
+        <v>9.718</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>1.675</v>
+        <v>1.299</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>-0.008999999999999999</v>
+        <v>-0.081</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>0.45</v>
+        <v>0.081</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Dummy (median)</t>
+          <t>Ridge</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>tuned</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr"/>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="n"/>
       <c r="E9" s="8" t="n">
-        <v>7.62</v>
+        <v>6.671</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.709</v>
+        <v>1.576</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>10.804</v>
+        <v>9.833</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>0.948</v>
+        <v>1.948</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>-0.113</v>
+        <v>-0.151</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>0.062</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="10">
@@ -3060,24 +3098,24 @@
           <t>Linear</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr"/>
+      <c r="D10" s="10" t="n"/>
       <c r="E10" s="8" t="n">
-        <v>7.851</v>
+        <v>6.812</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>1.759</v>
+        <v>1.65</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>10.286</v>
+        <v>10.143</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>1.797</v>
+        <v>2.029</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.221</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>0.485</v>
+        <v>0.437</v>
       </c>
     </row>
     <row r="11">
@@ -3096,24 +3134,24 @@
           <t>Linear</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr"/>
+      <c r="D11" s="10" t="n"/>
       <c r="E11" s="8" t="n">
-        <v>7.921</v>
+        <v>6.837</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1.712</v>
+        <v>1.555</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>10.301</v>
+        <v>15.552</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>1.809</v>
+        <v>11.436</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-4.286</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>0.483</v>
+        <v>8.380000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -3132,24 +3170,24 @@
           <t>Tree-based</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr"/>
+      <c r="D12" s="10" t="n"/>
       <c r="E12" s="8" t="n">
-        <v>8.747999999999999</v>
+        <v>8.643000000000001</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.426</v>
+        <v>1.612</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>12.483</v>
+        <v>12.673</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>0.466</v>
+        <v>1.888</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>-0.499</v>
+        <v>-0.884</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>0.134</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="13">
@@ -3168,30 +3206,30 @@
           <t>Reference</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr"/>
+      <c r="D13" s="10" t="n"/>
       <c r="E13" s="8" t="n">
-        <v>12.67</v>
+        <v>12.576</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>1.642</v>
+        <v>1.209</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>14.142</v>
+        <v>14.029</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>1.522</v>
+        <v>1.039</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>-0.995</v>
+        <v>-1.383</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>0.597</v>
+        <v>0.6870000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Note: Mean and standard deviation across folds, sorted by CV MAE. The champion is the default or tuned candidate with the lowest CV MAE.</t>
+          <t>Note: Mean and standard deviation across folds, sorted by CV MAE. The champion is the default or tuned candidate with the lowest hold-out MAE (sheet 6).</t>
         </is>
       </c>
     </row>
@@ -3245,10 +3283,10 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>5.869</v>
+        <v>5.43</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>6.247</v>
+        <v>5.752</v>
       </c>
     </row>
     <row r="4">
@@ -3258,10 +3296,10 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>8.263999999999999</v>
+        <v>7.949</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>8.944000000000001</v>
+        <v>8.622999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -3271,10 +3309,10 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>0.339</v>
+        <v>0.325</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>0.235</v>
+        <v>0.145</v>
       </c>
     </row>
     <row r="6">
@@ -3311,7 +3349,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Hold-out evaluation on the newest 45 approval days (2018-03-04 to 2018-04-17)</t>
+          <t>Hold-out evaluation on the newest 30 approval days (2018-03-19 to 2018-04-17)</t>
         </is>
       </c>
     </row>
@@ -3374,19 +3412,19 @@
         </is>
       </c>
       <c r="D3" s="12" t="n">
-        <v>6.103</v>
+        <v>5.847</v>
       </c>
       <c r="E3" s="12" t="n">
-        <v>8.795</v>
+        <v>8.193</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>0.34</v>
+        <v>0.249</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>4.159</v>
+        <v>4.346</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>-0.909</v>
+        <v>1.166</v>
       </c>
     </row>
     <row r="4">
@@ -3400,21 +3438,21 @@
           <t>default</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr"/>
+      <c r="C4" s="10" t="n"/>
       <c r="D4" s="8" t="n">
-        <v>6.403</v>
+        <v>6.022</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>9.124000000000001</v>
+        <v>8.237</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.289</v>
+        <v>0.241</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>4.36</v>
+        <v>4.759</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>-1.081</v>
+        <v>1.021</v>
       </c>
     </row>
     <row r="5">
@@ -3425,24 +3463,24 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr"/>
+          <t>tuned</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n"/>
       <c r="D5" s="8" t="n">
-        <v>6.469</v>
+        <v>6.022</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>9.047000000000001</v>
+        <v>8.237</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.301</v>
+        <v>0.241</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>4.58</v>
+        <v>4.757</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>-0.534</v>
+        <v>1.022</v>
       </c>
     </row>
     <row r="6">
@@ -3453,52 +3491,52 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr"/>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n"/>
       <c r="D6" s="8" t="n">
-        <v>6.506</v>
+        <v>6.024</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>9.048</v>
+        <v>8.237</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.301</v>
+        <v>0.241</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>4.718</v>
+        <v>4.759</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>-0.431</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>Dummy (median)</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr"/>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n"/>
       <c r="D7" s="8" t="n">
-        <v>6.629</v>
+        <v>6.63</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>8.823</v>
+        <v>9.646000000000001</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.335</v>
+        <v>-0.041</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>5.154</v>
+        <v>4</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>1.046</v>
+        <v>-2.11</v>
       </c>
     </row>
     <row r="8">
@@ -3512,27 +3550,27 @@
           <t>tuned</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr"/>
+      <c r="C8" s="10" t="n"/>
       <c r="D8" s="8" t="n">
-        <v>6.64</v>
+        <v>6.901</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>8.827999999999999</v>
+        <v>8.840999999999999</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.335</v>
+        <v>0.126</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>5.198</v>
+        <v>5.892</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>1.056</v>
+        <v>3.095</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -3540,77 +3578,77 @@
           <t>default</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr"/>
+      <c r="C9" s="10" t="n"/>
       <c r="D9" s="8" t="n">
-        <v>6.686</v>
+        <v>6.955</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>8.871</v>
+        <v>8.898999999999999</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.328</v>
+        <v>0.114</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>5.266</v>
+        <v>5.861</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>1.141</v>
+        <v>3.397</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Decision Tree</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr"/>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n"/>
       <c r="D10" s="8" t="n">
-        <v>6.811</v>
+        <v>7.084</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>9.045999999999999</v>
+        <v>9.114000000000001</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.301</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>5.353</v>
+        <v>6.067</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>1.07</v>
+        <v>3.132</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Dummy (median)</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr"/>
+          <t>tuned</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n"/>
       <c r="D11" s="8" t="n">
-        <v>7.958</v>
+        <v>7.404</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>11.084</v>
+        <v>9.545</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>-0.049</v>
+        <v>-0.019</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>6</v>
+        <v>6.093</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>-2.392</v>
+        <v>3.493</v>
       </c>
     </row>
     <row r="12">
@@ -3624,21 +3662,21 @@
           <t>default</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr"/>
+      <c r="C12" s="10" t="n"/>
       <c r="D12" s="8" t="n">
-        <v>9.047000000000001</v>
+        <v>9.255000000000001</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>12.785</v>
+        <v>13.074</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>-0.396</v>
+        <v>-0.912</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>6</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>1.731</v>
+        <v>3.468</v>
       </c>
     </row>
     <row r="13">
@@ -3652,27 +3690,27 @@
           <t>reference</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr"/>
+      <c r="C13" s="10" t="n"/>
       <c r="D13" s="8" t="n">
-        <v>11.315</v>
+        <v>11.867</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>13.15</v>
+        <v>13.55</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>-0.476</v>
+        <v>-1.053</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>8.193</v>
+        <v>9.744999999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Note: Models are fitted on the training part only. Bias = mean(predicted - actual). Predictions are clipped to 0-45 days.</t>
+          <t>Note: Models are fitted on the training part only. Bias = mean(predicted - actual). Predictions are clipped so that the implied lead time stays within 0-45 days.</t>
         </is>
       </c>
     </row>
@@ -3770,79 +3808,79 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Champion</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>re-selected monthly</t>
+          <t>tuned</t>
         </is>
       </c>
       <c r="C3" s="12" t="n">
-        <v>5.201</v>
+        <v>5.29</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>6.287</v>
+        <v>5.947</v>
       </c>
       <c r="E3" s="12" t="n">
-        <v>4.549</v>
+        <v>4.875</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>4.402</v>
+        <v>4.423</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>5.152</v>
+        <v>5.166</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>7.726</v>
+        <v>7.683</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.16</v>
+        <v>0.431</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>3.589</v>
+        <v>3.743</v>
       </c>
       <c r="K3" s="12" t="n">
-        <v>1.397</v>
+        <v>1.211</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>Champion</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
+          <t>re-selected monthly</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>5.201</v>
+        <v>5.96</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>6.287</v>
+        <v>7.187</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>4.549</v>
+        <v>4.875</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>4.402</v>
+        <v>4.423</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>5.152</v>
+        <v>5.674</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>7.726</v>
+        <v>8.06</v>
       </c>
       <c r="I4" s="8" t="n">
-        <v>0.16</v>
+        <v>0.374</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>3.589</v>
+        <v>4.263</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>1.397</v>
+        <v>2.295</v>
       </c>
     </row>
     <row r="5">
@@ -3857,31 +3895,31 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>4.97</v>
+        <v>5.484</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>6.79</v>
+        <v>6.312</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>6.946</v>
+        <v>6.549</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>4.86</v>
+        <v>5.666</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>5.901</v>
+        <v>6.001</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>8.27</v>
+        <v>8.077999999999999</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>0.038</v>
+        <v>0.371</v>
       </c>
       <c r="J5" s="8" t="n">
-        <v>4.476</v>
+        <v>4.875</v>
       </c>
       <c r="K5" s="8" t="n">
-        <v>2.015</v>
+        <v>2.705</v>
       </c>
     </row>
     <row r="6">
@@ -3892,35 +3930,35 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>tuned</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>5.547</v>
+        <v>5.492</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>6.501</v>
+        <v>6.312</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>6.922</v>
+        <v>6.548</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>4.927</v>
+        <v>5.665</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>5.983</v>
+        <v>6.003</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>8.226000000000001</v>
+        <v>8.077999999999999</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>0.048</v>
+        <v>0.371</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>4.675</v>
+        <v>4.877</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>2.441</v>
+        <v>2.711</v>
       </c>
     </row>
     <row r="7">
@@ -3931,230 +3969,230 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
+          <t>default</t>
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>5.641</v>
+        <v>5.538</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>6.402</v>
+        <v>6.317</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>6.986</v>
+        <v>6.544</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>5.249</v>
+        <v>5.656</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>6.071</v>
+        <v>6.013</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>8.214</v>
+        <v>8.077999999999999</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.051</v>
+        <v>0.371</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>4.877</v>
+        <v>4.891</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>2.745</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>tuned</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>6.076</v>
+        <v>5.814</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>7.47</v>
+        <v>6.917</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>5.611</v>
+        <v>6.35</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>5.29</v>
+        <v>5.069</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>6.158</v>
+        <v>6.063</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>8.346</v>
+        <v>8.247</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>0.02</v>
+        <v>0.345</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>4.784</v>
+        <v>4.898</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>3.25</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
+          <t>default</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>6.184</v>
+        <v>5.96</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>7.231</v>
+        <v>7.187</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>5.956</v>
+        <v>6.181</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>5.458</v>
+        <v>5.221</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>6.242</v>
+        <v>6.17</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>8.358000000000001</v>
+        <v>8.321</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>0.017</v>
+        <v>0.333</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>5.014</v>
+        <v>4.971</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>3.345</v>
+        <v>3.145</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Dummy (median)</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>default</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>6.45</v>
+        <v>5.807</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>6.698</v>
+        <v>7.485</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>5.943</v>
+        <v>7.027</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>5.954</v>
+        <v>5.214</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>6.281</v>
+        <v>6.408</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>8.529999999999999</v>
+        <v>8.606999999999999</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>-0.024</v>
+        <v>0.286</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>5</v>
+        <v>5.135</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>1.209</v>
+        <v>3.237</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>tuned</t>
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>6.259</v>
+        <v>5.955</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>7.273</v>
+        <v>7.667</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>6.24</v>
+        <v>7.039</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>5.516</v>
+        <v>5.332</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>6.354</v>
+        <v>6.526</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>8.49</v>
+        <v>8.773</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>-0.014</v>
+        <v>0.258</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>5.069</v>
+        <v>5.112</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>3.432</v>
+        <v>3.316</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Decision Tree</t>
+          <t>Dummy (median)</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>6.42</v>
+        <v>6.018</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>7.476</v>
+        <v>7.21</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>6.372</v>
+        <v>9.247999999999999</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>5.314</v>
+        <v>5.72</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>6.434</v>
+        <v>7.031</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>8.656000000000001</v>
+        <v>10.08</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>-0.054</v>
+        <v>0.021</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>5.082</v>
+        <v>5</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>3.425</v>
+        <v>1.296</v>
       </c>
     </row>
     <row r="13">
@@ -4169,31 +4207,31 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>8.327999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>9.961</v>
+        <v>10.167</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>7.373</v>
+        <v>7.686</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>7.726</v>
+        <v>7.542</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>8.401999999999999</v>
+        <v>8.429</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>12.494</v>
+        <v>12.543</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>-1.196</v>
+        <v>-0.516</v>
       </c>
       <c r="J13" s="8" t="n">
         <v>5</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>3.999</v>
+        <v>3.857</v>
       </c>
     </row>
     <row r="14">
@@ -4226,7 +4264,7 @@
         <v>16.525</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>-2.842</v>
+        <v>-1.631</v>
       </c>
       <c r="J14" s="8" t="n">
         <v>14</v>
@@ -4238,10 +4276,12 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Note: Each month: fit on the 2nd on that run date's 180-day window, score every order approved that month, evaluate at approval day + 45 days. Coverage: known capped targets at approval day + 45 days: 26,166/26,184 (99.93%). The Champion row uses the model re-selected at each run date.</t>
-        </is>
-      </c>
-    </row>
+          <t>Note: Each month: fit on the 2nd on that run date's 365-day window, score every order approved that month, evaluate at approval day + 45 days. Coverage: known targets at approval day + 45 days: 26,166/26,184 (99.93%). The Champion row uses the model re-selected at each run date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
@@ -4267,7 +4307,7 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Champion CV MAE (days)</t>
+          <t>Champion hold-out MAE (days)</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -4293,26 +4333,26 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>33847</v>
+        <v>52919</v>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
+          <t>LightGBM (default)</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>5.674</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>5.96</v>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
           <t>LightGBM (tuned)</t>
         </is>
       </c>
-      <c r="D20" s="8" t="n">
-        <v>5.226</v>
-      </c>
-      <c r="E20" s="8" t="n">
-        <v>5.201</v>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>Linear Regression (default)</t>
-        </is>
-      </c>
       <c r="G20" s="8" t="n">
-        <v>4.97</v>
+        <v>5.29</v>
       </c>
     </row>
     <row r="21">
@@ -4322,26 +4362,26 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>37072</v>
+        <v>58175</v>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
+          <t>LightGBM (default)</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>7.286</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>7.187</v>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
           <t>LightGBM (tuned)</t>
         </is>
       </c>
-      <c r="D21" s="8" t="n">
-        <v>5.587</v>
-      </c>
-      <c r="E21" s="8" t="n">
-        <v>6.287</v>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>LightGBM (tuned)</t>
-        </is>
-      </c>
       <c r="G21" s="8" t="n">
-        <v>6.287</v>
+        <v>5.947</v>
       </c>
     </row>
     <row r="22">
@@ -4351,7 +4391,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>39532</v>
+        <v>62841</v>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
@@ -4359,10 +4399,10 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>6.117</v>
+        <v>5.847</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>4.549</v>
+        <v>4.875</v>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
@@ -4370,7 +4410,7 @@
         </is>
       </c>
       <c r="G22" s="8" t="n">
-        <v>4.549</v>
+        <v>4.875</v>
       </c>
     </row>
     <row r="23">
@@ -4380,7 +4420,7 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>42621</v>
+        <v>67399</v>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
@@ -4388,10 +4428,10 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>6.136</v>
+        <v>4.796</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>4.402</v>
+        <v>4.423</v>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
@@ -4399,13 +4439,13 @@
         </is>
       </c>
       <c r="G23" s="8" t="n">
-        <v>4.402</v>
+        <v>4.423</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Note: Champion = lowest CV MAE on that run date's own window. Best in hindsight = lowest realised MAE that month among the candidates.</t>
+          <t>Note: Champion = lowest MAE on the hold-out of that run date's own window. Best in hindsight = lowest realised MAE that month among the candidates.</t>
         </is>
       </c>
     </row>
@@ -4464,14 +4504,14 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>route_type</t>
+          <t>promised_lead_days</t>
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>0.476</v>
+        <v>2.813</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>0.012</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="4">
@@ -4484,7 +4524,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>0.423</v>
+        <v>0.205</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>0.012</v>
@@ -4496,14 +4536,14 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>promised_lead_days</t>
+          <t>order_product_weight_g_sum</t>
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>0.343</v>
+        <v>0.054</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="6">
@@ -4512,14 +4552,14 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>seller_dist_km_min</t>
+          <t>order_product_volume_cm3_sum</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>0.261</v>
+        <v>0.045</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="7">
@@ -4528,14 +4568,14 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>seller_dist_km_median</t>
+          <t>orders_approved_prev_7d</t>
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>0.074</v>
+        <v>0.035</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>0.004</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="8">
@@ -4544,14 +4584,14 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>orders_approved_prev_7d</t>
+          <t>seller_dist_km_min</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>0.054</v>
+        <v>0.031</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>0.005</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="9">
@@ -4560,14 +4600,14 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>order_frieght_value_sum</t>
+          <t>seller_dist_km_median</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>0.037</v>
+        <v>0.018</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="10">
@@ -4576,14 +4616,14 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>order_product_volume_cm3_sum</t>
+          <t>payment_type_value_credit_card</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>0.03</v>
+        <v>0.016</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="11">
@@ -4592,11 +4632,11 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>seller_dist_km_mean</t>
+          <t>order_product_photos_mean</t>
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>0.028</v>
+        <v>0.016</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>0.001</v>
@@ -4608,14 +4648,14 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>order_product_weight_g_sum</t>
+          <t>order_pdt_price_sum</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>0.025</v>
+        <v>0.014</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Restore the 45-day gap before the regression hold-out and add a resampling experiment
- Hold-out split and the monthly champion selection again leave a 45-day
  gap after training and use only outcomes known at hold-out start, as in
  6ae5580. Training is 290 days; the hold-out stays at 30 days.
- New section: over- and undersampling late orders in the training data,
  compared on the hold-out and the April-July backtest.
- Findings, figures, tuning JSON and report tables regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/phase2/results/regression_report_tables.xlsx
+++ b/phase2/results/regression_report_tables.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Tuned hyperparameters" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Residuals by segment" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Derived late flag" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Resampling" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -501,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -560,7 +561,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>LightGBM (tuned), lowest hold-out MAE (5.847 days; CV MAE 5.624)</t>
+          <t>LightGBM (tuned), lowest hold-out MAE (5.354 days; CV MAE 5.244)</t>
         </is>
       </c>
     </row>
@@ -766,6 +767,30 @@
       <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Late flag derived from the regression output vs classifiers, same hold-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>12 Resampling</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Resampling the training data, LightGBM (tuned): hold-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>12 Resampling</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Resampling the training data, LightGBM (tuned): April-July 2018 backtest, pooled</t>
         </is>
       </c>
     </row>
@@ -869,7 +894,7 @@
         </is>
       </c>
       <c r="E3" s="8" t="n">
-        <v>6.837064070902182</v>
+        <v>6.044125632714844</v>
       </c>
       <c r="F3" s="10" t="n"/>
     </row>
@@ -890,13 +915,13 @@
         </is>
       </c>
       <c r="D4" s="13" t="n">
-        <v>0.08111308307896872</v>
+        <v>0.01</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>6.812111238922651</v>
+        <v>6.15842969474444</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>6.670931265188512</v>
+        <v>5.880321612611291</v>
       </c>
     </row>
     <row r="5">
@@ -919,10 +944,10 @@
         <v>200</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>8.642644390013142</v>
+        <v>8.020504142010939</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>5.912638205795114</v>
+        <v>5.491788669658639</v>
       </c>
     </row>
     <row r="6">
@@ -945,10 +970,10 @@
         <v>12</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>8.642644390013142</v>
+        <v>8.020504142010939</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>5.912638205795114</v>
+        <v>5.491788669658639</v>
       </c>
     </row>
     <row r="7">
@@ -971,10 +996,10 @@
         <v>200</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>5.885218329668307</v>
+        <v>5.530724311727721</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>5.708676430383172</v>
+        <v>5.311121771602226</v>
       </c>
     </row>
     <row r="8">
@@ -997,10 +1022,10 @@
         <v>60</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>5.885218329668307</v>
+        <v>5.530724311727721</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>5.708676430383172</v>
+        <v>5.311121771602226</v>
       </c>
     </row>
     <row r="9">
@@ -1023,10 +1048,10 @@
         <v>0.5</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>5.885218329668307</v>
+        <v>5.530724311727721</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>5.708676430383172</v>
+        <v>5.311121771602226</v>
       </c>
     </row>
     <row r="10">
@@ -1049,10 +1074,10 @@
         <v>16</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>5.885218329668307</v>
+        <v>5.530724311727721</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>5.708676430383172</v>
+        <v>5.311121771602226</v>
       </c>
     </row>
     <row r="11">
@@ -1075,10 +1100,10 @@
         <v>1</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>5.751597282021803</v>
+        <v>5.34193326913879</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>5.623849362046951</v>
+        <v>5.243782856967416</v>
       </c>
     </row>
     <row r="12">
@@ -1101,10 +1126,10 @@
         <v>1</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>5.751597282021803</v>
+        <v>5.34193326913879</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>5.623849362046951</v>
+        <v>5.243782856967416</v>
       </c>
     </row>
     <row r="13">
@@ -1129,10 +1154,10 @@
         </is>
       </c>
       <c r="E13" s="8" t="n">
-        <v>5.751597282021803</v>
+        <v>5.34193326913879</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>5.623849362046951</v>
+        <v>5.243782856967416</v>
       </c>
     </row>
     <row r="14">
@@ -1152,13 +1177,13 @@
         </is>
       </c>
       <c r="D14" s="13" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>5.751597282021803</v>
+        <v>5.34193326913879</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>5.623849362046951</v>
+        <v>5.243782856967416</v>
       </c>
     </row>
     <row r="15">
@@ -1181,10 +1206,10 @@
         <v>600</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>5.751597282021803</v>
+        <v>5.34193326913879</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>5.623849362046951</v>
+        <v>5.243782856967416</v>
       </c>
     </row>
     <row r="16">
@@ -1207,10 +1232,10 @@
         <v>100</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>5.751597282021803</v>
+        <v>5.34193326913879</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>5.623849362046951</v>
+        <v>5.243782856967416</v>
       </c>
     </row>
     <row r="17">
@@ -1233,10 +1258,10 @@
         <v>0.05</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>5.751597282021803</v>
+        <v>5.34193326913879</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>5.623849362046951</v>
+        <v>5.243782856967416</v>
       </c>
     </row>
     <row r="18">
@@ -1256,13 +1281,13 @@
         </is>
       </c>
       <c r="D18" s="13" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>5.751597282021803</v>
+        <v>5.34193326913879</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>5.623849362046951</v>
+        <v>5.243782856967416</v>
       </c>
     </row>
     <row r="19">
@@ -1346,13 +1371,13 @@
         <v>-10.104</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>-8.352</v>
+        <v>-12.524</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>1.752</v>
+        <v>-2.419</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>7.205</v>
+        <v>6.606</v>
       </c>
     </row>
     <row r="4">
@@ -1368,13 +1393,13 @@
         <v>-9.207000000000001</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>-8.94</v>
+        <v>-10.418</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>0.267</v>
+        <v>-1.211</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>3.813</v>
+        <v>3.485</v>
       </c>
     </row>
     <row r="5">
@@ -1390,13 +1415,13 @@
         <v>-18.957</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>-16.321</v>
+        <v>-18.455</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>2.635</v>
+        <v>0.502</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>3.294</v>
+        <v>2.254</v>
       </c>
     </row>
     <row r="6">
@@ -1460,13 +1485,13 @@
         <v>-9.821</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>-9.211</v>
+        <v>-11.005</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>0.611</v>
+        <v>-1.184</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>4.101</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="12">
@@ -1482,13 +1507,13 @@
         <v>-12.006</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>-8.954000000000001</v>
+        <v>-13.969</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>3.052</v>
+        <v>-1.963</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>9.728</v>
+        <v>8.625999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -1504,13 +1529,13 @@
         <v>-10.514</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>-8.983000000000001</v>
+        <v>-12.941</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>1.531</v>
+        <v>-2.427</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>5.629</v>
+        <v>5.082</v>
       </c>
     </row>
     <row r="14">
@@ -1526,13 +1551,13 @@
         <v>-12.047</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>-9.369999999999999</v>
+        <v>-13.055</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>2.677</v>
+        <v>-1.008</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>6.887</v>
+        <v>6.046</v>
       </c>
     </row>
     <row r="15">
@@ -1548,13 +1573,13 @@
         <v>-12.102</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>-9.829000000000001</v>
+        <v>-12.79</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>2.273</v>
+        <v>-0.6879999999999999</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>5.295</v>
+        <v>4.337</v>
       </c>
     </row>
     <row r="16">
@@ -1570,13 +1595,13 @@
         <v>-10.884</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>-7.013</v>
+        <v>-10.534</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>3.871</v>
+        <v>0.351</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>6.447</v>
+        <v>4.979</v>
       </c>
     </row>
     <row r="17">
@@ -1592,13 +1617,13 @@
         <v>-4.402</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>-5.56</v>
+        <v>-9.667</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>-1.158</v>
+        <v>-5.266</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>7.536</v>
+        <v>7.985</v>
       </c>
     </row>
     <row r="18">
@@ -1614,13 +1639,13 @@
         <v>-4.583</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>-5.967</v>
+        <v>-10.165</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>-1.384</v>
+        <v>-5.581</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>6.358</v>
+        <v>7.433</v>
       </c>
     </row>
     <row r="19">
@@ -1636,13 +1661,13 @@
         <v>-10.367</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>-6.296</v>
+        <v>-10.487</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>4.071</v>
+        <v>-0.12</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>6.082</v>
+        <v>4.432</v>
       </c>
     </row>
     <row r="20">
@@ -1658,13 +1683,13 @@
         <v>-8.24</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>-6.622</v>
+        <v>-11.099</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>1.618</v>
+        <v>-2.86</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>5.99</v>
+        <v>5.563</v>
       </c>
     </row>
     <row r="21">
@@ -1680,13 +1705,13 @@
         <v>-7.543</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>-7.381</v>
+        <v>-10.695</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>0.162</v>
+        <v>-3.152</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>7.559</v>
+        <v>7.474</v>
       </c>
     </row>
     <row r="22">
@@ -1702,13 +1727,13 @@
         <v>-1.92</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>-2.991</v>
+        <v>-8.991</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>-1.071</v>
+        <v>-7.071</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>9.477</v>
+        <v>10.498</v>
       </c>
     </row>
     <row r="23">
@@ -1793,22 +1818,22 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>0.896</v>
+        <v>0.899</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>0.432</v>
+        <v>0</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>0.106</v>
+        <v>0</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>0.707</v>
+        <v>0.637</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>0.25</v>
+        <v>0.155</v>
       </c>
     </row>
     <row r="4">
@@ -1818,22 +1843,22 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>0.414</v>
+        <v>0.676</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>0.128</v>
+        <v>0.139</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>0.832</v>
+        <v>0.43</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>0.222</v>
+        <v>0.21</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.676</v>
+        <v>0.6</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>0.208</v>
+        <v>0.157</v>
       </c>
     </row>
     <row r="5">
@@ -1843,22 +1868,22 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>0.673</v>
+        <v>0.768</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>0.185</v>
+        <v>0.207</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>0.662</v>
+        <v>0.462</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>0.29</v>
+        <v>0.286</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.705</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>0.208</v>
+        <v>0.194</v>
       </c>
     </row>
     <row r="6">
@@ -1868,22 +1893,22 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>0.391</v>
+        <v>0.747</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>0.132</v>
+        <v>0.205</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0.907</v>
+        <v>0.527</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>0.231</v>
+        <v>0.295</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.732</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>0.239</v>
+        <v>0.211</v>
       </c>
     </row>
     <row r="7">
@@ -1893,28 +1918,391 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.731</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>0.158</v>
+        <v>0.208</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>0.784</v>
+        <v>0.595</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>0.263</v>
+        <v>0.308</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.741</v>
+        <v>0.713</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.259</v>
+        <v>0.224</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Note: Regression-derived flag: predicted days from the promised date &gt; 0. Classifiers use a 0.5 threshold. Hold-out late rate: 10.06%. "v2 features" = the base classification feature set.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Resampling the training data, LightGBM (tuned): hold-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Training data</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Training rows</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Late orders in training (%)</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>MAE (days)</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>MAE, late orders (days)</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>MAE, other orders (days)</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Bias (days)</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Flagged late (%)</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Flag precision</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>Flag recall</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>Flag PR-AUC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>No resampling</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>45371</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>7.551</v>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>5.354</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>20.803</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>3.634</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>-1.93</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>0.155</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Oversample late orders</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>83890</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>7.847</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>12.429</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>7.337</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>4.363</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>18.534</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="J4" s="8" t="n">
+        <v>0.436</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>0.209</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Undersample other orders</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>6852</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>9.042999999999999</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>11.443</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>8.775</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>6.213</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>29.283</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>0.531</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>0.199</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Note: Late orders are those with a target above zero. Resampling balances late and other orders 1:1 in the training data only. Flag = predicted days above zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Resampling the training data, LightGBM (tuned): April-July 2018 backtest, pooled</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Training data</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>MAE (days)</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>MAE, late orders (days)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>MAE, other orders (days)</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Bias (days)</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Flagged late (%)</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Flag precision</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Flag recall</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Flag PR-AUC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>No resampling</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>5.141</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>20.963</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>4.193</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>1.122</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>0.317</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>0.277</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>0.118</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Oversample late orders</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>10.273</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>8.473000000000001</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>29.676</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Undersample other orders</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>10.847</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>12.833</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>10.729</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>9.113</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>33.964</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>0.124</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Note: Fitted on each run date's whole window with the same resampling, scored on that month's orders.</t>
         </is>
       </c>
     </row>
@@ -2323,14 +2711,14 @@
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>2018-03-18</t>
+          <t>2018-02-01</t>
         </is>
       </c>
       <c r="D3" s="7" t="n">
-        <v>55994</v>
+        <v>45371</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>-10.6</v>
+        <v>-11.44</v>
       </c>
     </row>
     <row r="4">
@@ -2359,7 +2747,7 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Note: The hold-out is the newest 30 approval days. Training uses every earlier approval day in the window.</t>
+          <t>Note: The hold-out is the newest 30 approval days. Training excludes the 45 days before it and outcomes not yet known at its start.</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2800,7 @@
         <v>4920</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>6631</v>
+        <v>5462</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
@@ -2421,11 +2809,11 @@
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>2017-09-03</t>
+          <t>2017-08-25</t>
         </is>
       </c>
       <c r="F10" s="8" t="n">
-        <v>-12.34</v>
+        <v>-12.62</v>
       </c>
     </row>
     <row r="11">
@@ -2433,23 +2821,23 @@
         <v>2</v>
       </c>
       <c r="B11" s="7" t="n">
-        <v>10579</v>
+        <v>9277</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>7151</v>
+        <v>5652</v>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>2017-09-04</t>
+          <t>2017-08-26</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>2017-10-22</t>
+          <t>2017-10-04</t>
         </is>
       </c>
       <c r="F11" s="8" t="n">
-        <v>-11.26</v>
+        <v>-11.24</v>
       </c>
     </row>
     <row r="12">
@@ -2457,23 +2845,23 @@
         <v>3</v>
       </c>
       <c r="B12" s="7" t="n">
-        <v>17137</v>
+        <v>14711</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>11010</v>
+        <v>5856</v>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>2017-10-23</t>
+          <t>2017-10-05</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>2017-12-10</t>
+          <t>2017-11-13</t>
         </is>
       </c>
       <c r="F12" s="8" t="n">
-        <v>-8.9</v>
+        <v>-10.82</v>
       </c>
     </row>
     <row r="13">
@@ -2481,23 +2869,23 @@
         <v>4</v>
       </c>
       <c r="B13" s="7" t="n">
-        <v>24334</v>
+        <v>20326</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>9717</v>
+        <v>10208</v>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>2017-12-11</t>
+          <t>2017-11-14</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>2018-01-28</t>
+          <t>2017-12-23</t>
         </is>
       </c>
       <c r="F13" s="8" t="n">
-        <v>-13.1</v>
+        <v>-9.369999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -2505,23 +2893,23 @@
         <v>5</v>
       </c>
       <c r="B14" s="7" t="n">
-        <v>35686</v>
+        <v>26090</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>11554</v>
+        <v>8262</v>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>2018-01-29</t>
+          <t>2017-12-24</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>2018-03-18</t>
+          <t>2018-02-01</t>
         </is>
       </c>
       <c r="F14" s="8" t="n">
-        <v>-7.38</v>
+        <v>-12.92</v>
       </c>
     </row>
     <row r="15">
@@ -2848,22 +3236,22 @@
         </is>
       </c>
       <c r="E3" s="12" t="n">
-        <v>5.624</v>
+        <v>5.244</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>0.974</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>8.856</v>
+        <v>8.441000000000001</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>1.062</v>
+        <v>1.079</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.098</v>
+        <v>0.103</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.081</v>
       </c>
     </row>
     <row r="4">
@@ -2884,22 +3272,22 @@
       </c>
       <c r="D4" s="10" t="n"/>
       <c r="E4" s="8" t="n">
-        <v>5.709</v>
+        <v>5.311</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.897</v>
+        <v>0.828</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>8.693</v>
+        <v>8.188000000000001</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>1.086</v>
+        <v>0.98</v>
       </c>
       <c r="I4" s="8" t="n">
-        <v>0.133</v>
+        <v>0.156</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="5">
@@ -2920,33 +3308,33 @@
       </c>
       <c r="D5" s="10" t="n"/>
       <c r="E5" s="8" t="n">
-        <v>5.752</v>
+        <v>5.342</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.877</v>
+        <v>0.839</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>8.622999999999999</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>1.043</v>
+        <v>0.907</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>0.145</v>
+        <v>0.169</v>
       </c>
       <c r="J5" s="8" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>tuned</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -2956,33 +3344,33 @@
       </c>
       <c r="D6" s="10" t="n"/>
       <c r="E6" s="8" t="n">
-        <v>5.885</v>
+        <v>5.492</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.917</v>
+        <v>0.875</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>8.675000000000001</v>
+        <v>8.364000000000001</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>1.038</v>
+        <v>1.025</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>0.135</v>
+        <v>0.119</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>0.082</v>
+        <v>0.06900000000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Decision Tree</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
+          <t>default</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -2992,19 +3380,19 @@
       </c>
       <c r="D7" s="10" t="n"/>
       <c r="E7" s="8" t="n">
-        <v>5.913</v>
+        <v>5.531</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.918</v>
+        <v>0.931</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>8.84</v>
+        <v>8.228</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>1.068</v>
+        <v>1.017</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.102</v>
+        <v>0.147</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>0.076</v>
@@ -3013,48 +3401,48 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Dummy (median)</t>
+          <t>Ridge</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>tuned</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Linear</t>
         </is>
       </c>
       <c r="D8" s="10" t="n"/>
       <c r="E8" s="8" t="n">
-        <v>6.586</v>
+        <v>5.88</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>1.036</v>
+        <v>1.476</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>9.718</v>
+        <v>9.037000000000001</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>1.299</v>
+        <v>1.792</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>-0.081</v>
+        <v>-0.043</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>0.081</v>
+        <v>0.293</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>Linear Regression</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
+          <t>default</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -3064,64 +3452,64 @@
       </c>
       <c r="D9" s="10" t="n"/>
       <c r="E9" s="8" t="n">
-        <v>6.671</v>
+        <v>6.044</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>1.576</v>
+        <v>1.546</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>9.833</v>
+        <v>15.678</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>1.948</v>
+        <v>12.608</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>-0.151</v>
+        <v>-5.003</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>0.42</v>
+        <v>9.813000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>Dummy (median)</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Linear</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="D10" s="10" t="n"/>
       <c r="E10" s="8" t="n">
-        <v>6.812</v>
+        <v>6.117</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>1.65</v>
+        <v>0.762</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>10.143</v>
+        <v>9.113</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>2.029</v>
+        <v>0.954</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>-0.221</v>
+        <v>-0.047</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>0.437</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Linear Regression</t>
+          <t>Ridge</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -3136,22 +3524,22 @@
       </c>
       <c r="D11" s="10" t="n"/>
       <c r="E11" s="8" t="n">
-        <v>6.837</v>
+        <v>6.158</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1.555</v>
+        <v>1.621</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>15.552</v>
+        <v>9.397</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>11.436</v>
+        <v>1.917</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>-4.286</v>
+        <v>-0.125</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>8.380000000000001</v>
+        <v>0.314</v>
       </c>
     </row>
     <row r="12">
@@ -3172,22 +3560,22 @@
       </c>
       <c r="D12" s="10" t="n"/>
       <c r="E12" s="8" t="n">
-        <v>8.643000000000001</v>
+        <v>8.021000000000001</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>1.612</v>
+        <v>1.106</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>12.673</v>
+        <v>11.921</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>1.888</v>
+        <v>1.116</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>-0.884</v>
+        <v>-0.796</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>0.52</v>
+        <v>0.102</v>
       </c>
     </row>
     <row r="13">
@@ -3208,22 +3596,22 @@
       </c>
       <c r="D13" s="10" t="n"/>
       <c r="E13" s="8" t="n">
-        <v>12.576</v>
+        <v>12.904</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>1.209</v>
+        <v>0.832</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>14.029</v>
+        <v>14.292</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>1.039</v>
+        <v>0.731</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>-1.383</v>
+        <v>-1.651</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>0.6870000000000001</v>
+        <v>0.537</v>
       </c>
     </row>
     <row r="14">
@@ -3283,10 +3671,10 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>5.43</v>
+        <v>5.154</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>5.752</v>
+        <v>5.342</v>
       </c>
     </row>
     <row r="4">
@@ -3296,10 +3684,10 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>7.949</v>
+        <v>7.712</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>8.622999999999999</v>
+        <v>8.119999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -3309,10 +3697,10 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>0.325</v>
+        <v>0.291</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>0.145</v>
+        <v>0.169</v>
       </c>
     </row>
     <row r="6">
@@ -3412,25 +3800,25 @@
         </is>
       </c>
       <c r="D3" s="12" t="n">
-        <v>5.847</v>
+        <v>5.354</v>
       </c>
       <c r="E3" s="12" t="n">
-        <v>8.193</v>
+        <v>8.44</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>0.249</v>
+        <v>0.203</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>4.346</v>
+        <v>3.202</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>1.166</v>
+        <v>-1.93</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Linear Regression</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -3440,47 +3828,47 @@
       </c>
       <c r="C4" s="10" t="n"/>
       <c r="D4" s="8" t="n">
-        <v>6.022</v>
+        <v>5.569</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>8.237</v>
+        <v>8.279</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.241</v>
+        <v>0.234</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>4.759</v>
+        <v>3.759</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>1.021</v>
+        <v>-0.623</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>Linear Regression</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
+          <t>default</t>
         </is>
       </c>
       <c r="C5" s="10" t="n"/>
       <c r="D5" s="8" t="n">
-        <v>6.022</v>
+        <v>5.585</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>8.237</v>
+        <v>8.340999999999999</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.241</v>
+        <v>0.222</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>4.757</v>
+        <v>3.787</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>1.022</v>
+        <v>-0.9330000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -3491,52 +3879,52 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>tuned</t>
         </is>
       </c>
       <c r="C6" s="10" t="n"/>
       <c r="D6" s="8" t="n">
-        <v>6.024</v>
+        <v>5.585</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>8.237</v>
+        <v>8.34</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.241</v>
+        <v>0.222</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>4.759</v>
+        <v>3.787</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>1.03</v>
+        <v>-0.928</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Dummy (median)</t>
+          <t>Ridge</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>default</t>
         </is>
       </c>
       <c r="C7" s="10" t="n"/>
       <c r="D7" s="8" t="n">
-        <v>6.63</v>
+        <v>5.602</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>9.646000000000001</v>
+        <v>8.305</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>-0.041</v>
+        <v>0.229</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>4</v>
+        <v>3.856</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>-2.11</v>
+        <v>-0.745</v>
       </c>
     </row>
     <row r="8">
@@ -3552,25 +3940,25 @@
       </c>
       <c r="C8" s="10" t="n"/>
       <c r="D8" s="8" t="n">
-        <v>6.901</v>
+        <v>5.669</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>8.840999999999999</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.126</v>
+        <v>0.215</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>5.892</v>
+        <v>3.903</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>3.095</v>
+        <v>-0.633</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -3580,75 +3968,75 @@
       </c>
       <c r="C9" s="10" t="n"/>
       <c r="D9" s="8" t="n">
-        <v>6.955</v>
+        <v>5.729</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>8.898999999999999</v>
+        <v>8.433</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.114</v>
+        <v>0.205</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>5.861</v>
+        <v>3.925</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>3.397</v>
+        <v>-0.553</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>tuned</t>
         </is>
       </c>
       <c r="C10" s="10" t="n"/>
       <c r="D10" s="8" t="n">
-        <v>7.084</v>
+        <v>5.767</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>9.114000000000001</v>
+        <v>8.542</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.184</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>6.067</v>
+        <v>3.838</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>3.132</v>
+        <v>-0.474</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Decision Tree</t>
+          <t>Dummy (median)</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>tuned</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="C11" s="10" t="n"/>
       <c r="D11" s="8" t="n">
-        <v>7.404</v>
+        <v>6.733</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>9.545</v>
+        <v>9.864000000000001</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>-0.019</v>
+        <v>-0.08799999999999999</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>6.093</v>
+        <v>5</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>3.493</v>
+        <v>-3.022</v>
       </c>
     </row>
     <row r="12">
@@ -3664,19 +4052,19 @@
       </c>
       <c r="C12" s="10" t="n"/>
       <c r="D12" s="8" t="n">
-        <v>9.255000000000001</v>
+        <v>8.269</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>13.074</v>
+        <v>12.308</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>-0.912</v>
+        <v>-0.694</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>3.468</v>
+        <v>0.323</v>
       </c>
     </row>
     <row r="13">
@@ -3817,31 +4205,31 @@
         </is>
       </c>
       <c r="C3" s="12" t="n">
-        <v>5.29</v>
+        <v>5.131</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>5.947</v>
+        <v>5.872</v>
       </c>
       <c r="E3" s="12" t="n">
-        <v>4.875</v>
+        <v>4.987</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>4.423</v>
+        <v>4.466</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>5.166</v>
+        <v>5.141</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>7.683</v>
+        <v>7.667</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>0.431</v>
+        <v>0.434</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>3.743</v>
+        <v>3.701</v>
       </c>
       <c r="K3" s="12" t="n">
-        <v>1.211</v>
+        <v>1.122</v>
       </c>
     </row>
     <row r="4">
@@ -3856,31 +4244,31 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>5.96</v>
+        <v>5.131</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>7.187</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>4.875</v>
+        <v>4.987</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>4.423</v>
+        <v>4.466</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>5.674</v>
+        <v>5.496</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>8.06</v>
+        <v>7.991</v>
       </c>
       <c r="I4" s="8" t="n">
-        <v>0.374</v>
+        <v>0.385</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>4.263</v>
+        <v>3.974</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>2.295</v>
+        <v>1.852</v>
       </c>
     </row>
     <row r="5">
@@ -3934,19 +4322,19 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>5.492</v>
+        <v>5.485</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>6.312</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>6.548</v>
+        <v>6.549</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>5.665</v>
+        <v>5.666</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>6.003</v>
+        <v>6.001</v>
       </c>
       <c r="H6" s="8" t="n">
         <v>8.077999999999999</v>
@@ -3955,10 +4343,10 @@
         <v>0.371</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>4.877</v>
+        <v>4.874</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>2.711</v>
+        <v>2.707</v>
       </c>
     </row>
     <row r="7">
@@ -4337,14 +4725,14 @@
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>LightGBM (default)</t>
+          <t>LightGBM (tuned)</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>5.674</v>
+        <v>5.682</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>5.96</v>
+        <v>5.131</v>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
@@ -4352,7 +4740,7 @@
         </is>
       </c>
       <c r="G20" s="8" t="n">
-        <v>5.29</v>
+        <v>5.131</v>
       </c>
     </row>
     <row r="21">
@@ -4370,7 +4758,7 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>7.286</v>
+        <v>7.495</v>
       </c>
       <c r="E21" s="8" t="n">
         <v>7.187</v>
@@ -4381,7 +4769,7 @@
         </is>
       </c>
       <c r="G21" s="8" t="n">
-        <v>5.947</v>
+        <v>5.872</v>
       </c>
     </row>
     <row r="22">
@@ -4399,10 +4787,10 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>5.847</v>
+        <v>5.354</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>4.875</v>
+        <v>4.987</v>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
@@ -4410,7 +4798,7 @@
         </is>
       </c>
       <c r="G22" s="8" t="n">
-        <v>4.875</v>
+        <v>4.987</v>
       </c>
     </row>
     <row r="23">
@@ -4428,10 +4816,10 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>4.796</v>
+        <v>5.759</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>4.423</v>
+        <v>4.466</v>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
@@ -4439,7 +4827,7 @@
         </is>
       </c>
       <c r="G23" s="8" t="n">
-        <v>4.423</v>
+        <v>4.466</v>
       </c>
     </row>
     <row r="24">
@@ -4508,10 +4896,10 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>2.813</v>
+        <v>2.809</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>0.024</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="4">
@@ -4524,10 +4912,10 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>0.205</v>
+        <v>0.28</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>0.012</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="5">
@@ -4536,14 +4924,14 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>order_product_weight_g_sum</t>
+          <t>seller_dist_km_min</t>
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>0.054</v>
+        <v>0.194</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="6">
@@ -4552,11 +4940,11 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>order_product_volume_cm3_sum</t>
+          <t>route_type</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>0.045</v>
+        <v>0.048</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>0.003</v>
@@ -4568,14 +4956,14 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>orders_approved_prev_7d</t>
+          <t>order_frieght_value_sum</t>
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>0.035</v>
+        <v>0.04</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>0.007</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="8">
@@ -4584,14 +4972,14 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>seller_dist_km_min</t>
+          <t>order_product_volume_cm3_sum</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>0.031</v>
+        <v>0.032</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>0.012</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="9">
@@ -4600,14 +4988,14 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>seller_dist_km_median</t>
+          <t>order_approved_day_of_week</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>0.018</v>
+        <v>0.029</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="10">
@@ -4616,11 +5004,11 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>payment_type_value_credit_card</t>
+          <t>seller_dist_km_median</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>0.016</v>
+        <v>0.029</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>0.002</v>
@@ -4632,14 +5020,14 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>order_product_photos_mean</t>
+          <t>seller_dist_km_max</t>
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>0.016</v>
+        <v>0.028</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="12">
@@ -4648,14 +5036,14 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>order_pdt_price_sum</t>
+          <t>order_product_weight_g_sum</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>0.014</v>
+        <v>0.025</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="13">

</xml_diff>